<commit_message>
problemas docn mobile pppp
</commit_message>
<xml_diff>
--- a/scripts/.tmp/consolidado-test.xlsx
+++ b/scripts/.tmp/consolidado-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121944EB-68AE-4CE1-8C80-B49289578493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49775DE-810D-4758-A059-F713516FBF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -1021,7 +1021,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="227">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1409,166 +1409,6 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1584,41 +1424,20 @@
     <xf numFmtId="1" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1630,6 +1449,166 @@
     </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1972,7 +1951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W113"/>
+  <dimension ref="A1:W112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -2001,12 +1980,12 @@
       </c>
       <c r="B1" s="112" t="inlineStr">
         <is>
-          <t xml:space="preserve">JUAN PEREZ</t>
+          <t xml:space="preserve">ANA</t>
         </is>
       </c>
       <c r="C1" s="120" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA LOPEZ</t>
+          <t xml:space="preserve">BOB</t>
         </is>
       </c>
       <c r="D1" s="120"/>
@@ -2081,7 +2060,7 @@
       <c r="S3" s="120"/>
       <c r="T3" s="120"/>
       <c r="U3" s="110"/>
-      <c r="V3" s="224"/>
+      <c r="V3" s="163"/>
       <c r="W3" s="116"/>
     </row>
     <row r="4" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2108,7 +2087,7 @@
       <c r="S4" s="120"/>
       <c r="T4" s="120"/>
       <c r="U4" s="110"/>
-      <c r="V4" s="224"/>
+      <c r="V4" s="163"/>
       <c r="W4" s="116"/>
     </row>
     <row r="5" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2117,12 +2096,12 @@
       </c>
       <c r="B5" s="129" t="inlineStr">
         <is>
-          <t xml:space="preserve">12345</t>
+          <t xml:space="preserve">111</t>
         </is>
       </c>
       <c r="C5" s="129" t="inlineStr">
         <is>
-          <t xml:space="preserve">67890</t>
+          <t xml:space="preserve">222</t>
         </is>
       </c>
       <c r="D5" s="129"/>
@@ -2151,10 +2130,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="120">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C6" s="120">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="120"/>
       <c r="E6" s="120"/>
@@ -2177,436 +2156,432 @@
       <c r="V6" s="111"/>
       <c r="W6" s="111"/>
     </row>
-    <row r="7" spans="1:23" s="213" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" s="45" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="122" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="225">
-        <v>1000000</v>
-      </c>
-      <c r="C7" s="225">
-        <v>1000000</v>
-      </c>
-      <c r="D7" s="225"/>
-      <c r="E7" s="225"/>
-      <c r="F7" s="225"/>
-      <c r="G7" s="225"/>
-      <c r="H7" s="225"/>
-      <c r="I7" s="225"/>
-      <c r="J7" s="225"/>
-      <c r="K7" s="225"/>
-      <c r="L7" s="225"/>
-      <c r="M7" s="225"/>
-      <c r="N7" s="225"/>
-      <c r="O7" s="225"/>
-      <c r="P7" s="225"/>
-      <c r="Q7" s="225"/>
-      <c r="R7" s="211"/>
-      <c r="S7" s="211"/>
-      <c r="T7" s="211"/>
-      <c r="U7" s="212"/>
-      <c r="V7" s="212"/>
-      <c r="W7" s="212"/>
-    </row>
-    <row r="8" spans="1:23" s="221" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="210"/>
-      <c r="B8" s="212"/>
-      <c r="C8" s="214"/>
-      <c r="D8" s="212"/>
-      <c r="E8" s="214"/>
-      <c r="F8" s="215"/>
-      <c r="G8" s="214"/>
-      <c r="H8" s="212"/>
-      <c r="I8" s="214"/>
-      <c r="J8" s="212"/>
-      <c r="K8" s="214"/>
-      <c r="L8" s="215"/>
-      <c r="M8" s="214"/>
-      <c r="N8" s="215"/>
-      <c r="O8" s="214"/>
-      <c r="P8" s="216"/>
-      <c r="Q8" s="214"/>
-      <c r="R8" s="216"/>
-      <c r="S8" s="214"/>
-      <c r="T8" s="216"/>
-      <c r="U8" s="214"/>
-      <c r="V8" s="215"/>
-      <c r="W8" s="214"/>
-    </row>
-    <row r="9" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="217" t="s">
+      <c r="B7" s="164">
+        <v>500000</v>
+      </c>
+      <c r="C7" s="164">
+        <v>500000</v>
+      </c>
+      <c r="D7" s="164"/>
+      <c r="E7" s="164"/>
+      <c r="F7" s="164"/>
+      <c r="G7" s="164"/>
+      <c r="H7" s="164"/>
+      <c r="I7" s="164"/>
+      <c r="J7" s="164"/>
+      <c r="K7" s="164"/>
+      <c r="L7" s="164"/>
+      <c r="M7" s="164"/>
+      <c r="N7" s="164"/>
+      <c r="O7" s="164"/>
+      <c r="P7" s="164"/>
+      <c r="Q7" s="164"/>
+      <c r="R7" s="156"/>
+      <c r="S7" s="156"/>
+      <c r="T7" s="156"/>
+      <c r="U7" s="157"/>
+      <c r="V7" s="157"/>
+      <c r="W7" s="157"/>
+    </row>
+    <row r="8" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="112"/>
+      <c r="B8" s="157"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="157"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="157"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="157"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="110"/>
+      <c r="M8" s="111"/>
+      <c r="N8" s="110"/>
+      <c r="O8" s="111"/>
+      <c r="P8" s="158"/>
+      <c r="Q8" s="111"/>
+      <c r="R8" s="158"/>
+      <c r="S8" s="111"/>
+      <c r="T8" s="158"/>
+      <c r="U8" s="111"/>
+      <c r="V8" s="110"/>
+      <c r="W8" s="111"/>
+    </row>
+    <row r="9" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="113" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="226">
-        <v>450000</v>
-      </c>
-      <c r="C9" s="226">
-        <v>450000</v>
-      </c>
-      <c r="D9" s="226"/>
-      <c r="E9" s="212"/>
-      <c r="F9" s="215"/>
-      <c r="G9" s="212"/>
-      <c r="H9" s="215"/>
-      <c r="I9" s="212"/>
-      <c r="J9" s="215"/>
-      <c r="K9" s="212"/>
-      <c r="L9" s="215"/>
-      <c r="M9" s="212"/>
-      <c r="N9" s="215"/>
-      <c r="O9" s="212"/>
-      <c r="P9" s="216"/>
-      <c r="Q9" s="212"/>
-      <c r="R9" s="216"/>
-      <c r="S9" s="218"/>
-      <c r="T9" s="218"/>
-      <c r="U9" s="212"/>
-      <c r="V9" s="215"/>
-      <c r="W9" s="212"/>
-    </row>
-    <row r="10" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="217" t="s">
+      <c r="B9" s="165">
+        <v>90000</v>
+      </c>
+      <c r="C9" s="165">
+        <v>90000</v>
+      </c>
+      <c r="D9" s="165"/>
+      <c r="E9" s="157"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="157"/>
+      <c r="H9" s="110"/>
+      <c r="I9" s="157"/>
+      <c r="J9" s="110"/>
+      <c r="K9" s="157"/>
+      <c r="L9" s="110"/>
+      <c r="M9" s="157"/>
+      <c r="N9" s="110"/>
+      <c r="O9" s="157"/>
+      <c r="P9" s="158"/>
+      <c r="Q9" s="157"/>
+      <c r="R9" s="158"/>
+      <c r="S9" s="159"/>
+      <c r="T9" s="159"/>
+      <c r="U9" s="157"/>
+      <c r="V9" s="110"/>
+      <c r="W9" s="157"/>
+    </row>
+    <row r="10" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="113" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="226">
-        <v>50000</v>
-      </c>
-      <c r="C10" s="226">
-        <v>50000</v>
-      </c>
-      <c r="D10" s="226"/>
-      <c r="E10" s="212"/>
-      <c r="F10" s="215"/>
-      <c r="G10" s="212"/>
-      <c r="H10" s="215"/>
-      <c r="I10" s="212"/>
-      <c r="J10" s="215"/>
-      <c r="K10" s="212"/>
-      <c r="L10" s="215"/>
-      <c r="M10" s="212"/>
-      <c r="N10" s="215"/>
-      <c r="O10" s="212"/>
-      <c r="P10" s="216"/>
-      <c r="Q10" s="212"/>
-      <c r="R10" s="216"/>
-      <c r="S10" s="218"/>
-      <c r="T10" s="218"/>
-      <c r="U10" s="212"/>
-      <c r="V10" s="215"/>
-      <c r="W10" s="212"/>
-    </row>
-    <row r="11" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="217" t="s">
+      <c r="B10" s="165">
+        <v>10000</v>
+      </c>
+      <c r="C10" s="165">
+        <v>10000</v>
+      </c>
+      <c r="D10" s="165"/>
+      <c r="E10" s="157"/>
+      <c r="F10" s="110"/>
+      <c r="G10" s="157"/>
+      <c r="H10" s="110"/>
+      <c r="I10" s="157"/>
+      <c r="J10" s="110"/>
+      <c r="K10" s="157"/>
+      <c r="L10" s="110"/>
+      <c r="M10" s="157"/>
+      <c r="N10" s="110"/>
+      <c r="O10" s="157"/>
+      <c r="P10" s="158"/>
+      <c r="Q10" s="157"/>
+      <c r="R10" s="158"/>
+      <c r="S10" s="159"/>
+      <c r="T10" s="159"/>
+      <c r="U10" s="157"/>
+      <c r="V10" s="110"/>
+      <c r="W10" s="157"/>
+    </row>
+    <row r="11" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="226">
-        <v>300000</v>
-      </c>
-      <c r="C11" s="226">
-        <v>300000</v>
-      </c>
-      <c r="D11" s="226"/>
-      <c r="E11" s="212"/>
-      <c r="F11" s="215"/>
-      <c r="G11" s="212"/>
-      <c r="H11" s="215"/>
-      <c r="I11" s="212"/>
-      <c r="J11" s="215"/>
-      <c r="K11" s="212"/>
-      <c r="L11" s="215"/>
-      <c r="M11" s="212"/>
-      <c r="N11" s="215"/>
-      <c r="O11" s="212"/>
-      <c r="P11" s="216"/>
-      <c r="Q11" s="212"/>
-      <c r="R11" s="216"/>
-      <c r="S11" s="218"/>
-      <c r="T11" s="218"/>
-      <c r="U11" s="212"/>
-      <c r="V11" s="215"/>
-      <c r="W11" s="212"/>
-    </row>
-    <row r="12" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="217" t="s">
+      <c r="B11" s="165"/>
+      <c r="C11" s="165"/>
+      <c r="D11" s="165"/>
+      <c r="E11" s="157"/>
+      <c r="F11" s="110"/>
+      <c r="G11" s="157"/>
+      <c r="H11" s="110"/>
+      <c r="I11" s="157"/>
+      <c r="J11" s="110"/>
+      <c r="K11" s="157"/>
+      <c r="L11" s="110"/>
+      <c r="M11" s="157"/>
+      <c r="N11" s="110"/>
+      <c r="O11" s="157"/>
+      <c r="P11" s="158"/>
+      <c r="Q11" s="157"/>
+      <c r="R11" s="158"/>
+      <c r="S11" s="159"/>
+      <c r="T11" s="159"/>
+      <c r="U11" s="157"/>
+      <c r="V11" s="110"/>
+      <c r="W11" s="157"/>
+    </row>
+    <row r="12" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="113" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="226"/>
-      <c r="C12" s="226"/>
-      <c r="D12" s="226"/>
-      <c r="E12" s="212"/>
-      <c r="F12" s="215"/>
-      <c r="G12" s="212"/>
-      <c r="H12" s="215"/>
-      <c r="I12" s="212"/>
-      <c r="J12" s="215"/>
-      <c r="K12" s="212"/>
-      <c r="L12" s="215"/>
-      <c r="M12" s="212"/>
-      <c r="N12" s="215"/>
-      <c r="O12" s="212"/>
-      <c r="P12" s="216"/>
-      <c r="Q12" s="212"/>
-      <c r="R12" s="216"/>
-      <c r="S12" s="218"/>
-      <c r="T12" s="218"/>
-      <c r="U12" s="212"/>
-      <c r="V12" s="215"/>
-      <c r="W12" s="212"/>
-    </row>
-    <row r="13" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="217" t="s">
+      <c r="B12" s="165"/>
+      <c r="C12" s="165"/>
+      <c r="D12" s="165"/>
+      <c r="E12" s="157"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="157"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="157"/>
+      <c r="J12" s="110"/>
+      <c r="K12" s="157"/>
+      <c r="L12" s="110"/>
+      <c r="M12" s="157"/>
+      <c r="N12" s="110"/>
+      <c r="O12" s="157"/>
+      <c r="P12" s="158"/>
+      <c r="Q12" s="157"/>
+      <c r="R12" s="158"/>
+      <c r="S12" s="159"/>
+      <c r="T12" s="159"/>
+      <c r="U12" s="157"/>
+      <c r="V12" s="110"/>
+      <c r="W12" s="157"/>
+    </row>
+    <row r="13" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="226"/>
-      <c r="C13" s="226"/>
-      <c r="D13" s="226"/>
-      <c r="E13" s="212"/>
-      <c r="F13" s="215"/>
-      <c r="G13" s="212"/>
-      <c r="H13" s="215"/>
-      <c r="I13" s="212"/>
-      <c r="J13" s="215"/>
-      <c r="K13" s="212"/>
-      <c r="L13" s="215"/>
-      <c r="M13" s="212"/>
-      <c r="N13" s="215"/>
-      <c r="O13" s="212"/>
-      <c r="P13" s="216"/>
-      <c r="Q13" s="212"/>
-      <c r="R13" s="216"/>
-      <c r="S13" s="218"/>
-      <c r="T13" s="218"/>
-      <c r="U13" s="212"/>
-      <c r="V13" s="215"/>
-      <c r="W13" s="212"/>
-    </row>
-    <row r="14" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="217" t="s">
+      <c r="B13" s="165"/>
+      <c r="C13" s="165"/>
+      <c r="D13" s="165"/>
+      <c r="E13" s="157"/>
+      <c r="F13" s="110"/>
+      <c r="G13" s="157"/>
+      <c r="H13" s="110"/>
+      <c r="I13" s="157"/>
+      <c r="J13" s="110"/>
+      <c r="K13" s="157"/>
+      <c r="L13" s="110"/>
+      <c r="M13" s="157"/>
+      <c r="N13" s="110"/>
+      <c r="O13" s="157"/>
+      <c r="P13" s="158"/>
+      <c r="Q13" s="157"/>
+      <c r="R13" s="158"/>
+      <c r="S13" s="159"/>
+      <c r="T13" s="159"/>
+      <c r="U13" s="157"/>
+      <c r="V13" s="110"/>
+      <c r="W13" s="157"/>
+    </row>
+    <row r="14" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="226"/>
-      <c r="C14" s="226"/>
-      <c r="D14" s="226"/>
-      <c r="E14" s="212"/>
-      <c r="F14" s="215"/>
-      <c r="G14" s="212"/>
-      <c r="H14" s="215"/>
-      <c r="I14" s="212"/>
-      <c r="J14" s="215"/>
-      <c r="K14" s="212"/>
-      <c r="L14" s="215"/>
-      <c r="M14" s="212"/>
-      <c r="N14" s="215"/>
-      <c r="O14" s="212"/>
-      <c r="P14" s="216"/>
-      <c r="Q14" s="212"/>
-      <c r="R14" s="216"/>
-      <c r="S14" s="218"/>
-      <c r="T14" s="218"/>
-      <c r="U14" s="212"/>
-      <c r="V14" s="215"/>
-      <c r="W14" s="212"/>
-    </row>
-    <row r="15" spans="1:23" s="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="217" t="s">
+      <c r="B14" s="165"/>
+      <c r="C14" s="165"/>
+      <c r="D14" s="165"/>
+      <c r="E14" s="157"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="157"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="157"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="157"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="157"/>
+      <c r="N14" s="110"/>
+      <c r="O14" s="157"/>
+      <c r="P14" s="158"/>
+      <c r="Q14" s="157"/>
+      <c r="R14" s="158"/>
+      <c r="S14" s="159"/>
+      <c r="T14" s="159"/>
+      <c r="U14" s="157"/>
+      <c r="V14" s="110"/>
+      <c r="W14" s="157"/>
+    </row>
+    <row r="15" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="113" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="226"/>
-      <c r="C15" s="226"/>
-      <c r="D15" s="226"/>
-      <c r="E15" s="212"/>
-      <c r="F15" s="215"/>
-      <c r="G15" s="212"/>
-      <c r="H15" s="215"/>
-      <c r="I15" s="212"/>
-      <c r="J15" s="215"/>
-      <c r="K15" s="212"/>
-      <c r="L15" s="215"/>
-      <c r="M15" s="212"/>
-      <c r="N15" s="215"/>
-      <c r="O15" s="212"/>
-      <c r="P15" s="216"/>
-      <c r="Q15" s="212"/>
-      <c r="R15" s="216"/>
-      <c r="S15" s="218"/>
-      <c r="T15" s="218"/>
-      <c r="U15" s="212"/>
-      <c r="V15" s="215"/>
-      <c r="W15" s="212"/>
-    </row>
-    <row r="16" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="217" t="s">
+      <c r="B15" s="165"/>
+      <c r="C15" s="165"/>
+      <c r="D15" s="165"/>
+      <c r="E15" s="157"/>
+      <c r="F15" s="110"/>
+      <c r="G15" s="157"/>
+      <c r="H15" s="110"/>
+      <c r="I15" s="157"/>
+      <c r="J15" s="110"/>
+      <c r="K15" s="157"/>
+      <c r="L15" s="110"/>
+      <c r="M15" s="157"/>
+      <c r="N15" s="110"/>
+      <c r="O15" s="157"/>
+      <c r="P15" s="158"/>
+      <c r="Q15" s="157"/>
+      <c r="R15" s="158"/>
+      <c r="S15" s="159"/>
+      <c r="T15" s="159"/>
+      <c r="U15" s="157"/>
+      <c r="V15" s="110"/>
+      <c r="W15" s="157"/>
+    </row>
+    <row r="16" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="226"/>
-      <c r="C16" s="226"/>
-      <c r="D16" s="226"/>
-      <c r="E16" s="212"/>
-      <c r="F16" s="215"/>
-      <c r="G16" s="212"/>
-      <c r="H16" s="215"/>
-      <c r="I16" s="219"/>
-      <c r="J16" s="215"/>
-      <c r="K16" s="219"/>
-      <c r="L16" s="215"/>
-      <c r="M16" s="212"/>
-      <c r="N16" s="215"/>
-      <c r="O16" s="212"/>
-      <c r="P16" s="216"/>
-      <c r="Q16" s="212"/>
-      <c r="R16" s="216"/>
-      <c r="S16" s="218"/>
-      <c r="T16" s="218"/>
-      <c r="U16" s="212"/>
-      <c r="V16" s="215"/>
-      <c r="W16" s="212"/>
-    </row>
-    <row r="17" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="217" t="s">
+      <c r="B16" s="165"/>
+      <c r="C16" s="165"/>
+      <c r="D16" s="165"/>
+      <c r="E16" s="157"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="110"/>
+      <c r="I16" s="160"/>
+      <c r="J16" s="110"/>
+      <c r="K16" s="160"/>
+      <c r="L16" s="110"/>
+      <c r="M16" s="157"/>
+      <c r="N16" s="110"/>
+      <c r="O16" s="157"/>
+      <c r="P16" s="158"/>
+      <c r="Q16" s="157"/>
+      <c r="R16" s="158"/>
+      <c r="S16" s="159"/>
+      <c r="T16" s="159"/>
+      <c r="U16" s="157"/>
+      <c r="V16" s="110"/>
+      <c r="W16" s="157"/>
+    </row>
+    <row r="17" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="226"/>
-      <c r="C17" s="226"/>
-      <c r="D17" s="226"/>
-      <c r="E17" s="212"/>
-      <c r="F17" s="215"/>
-      <c r="G17" s="212"/>
-      <c r="H17" s="215"/>
-      <c r="I17" s="219"/>
-      <c r="J17" s="215"/>
-      <c r="K17" s="212"/>
-      <c r="L17" s="215"/>
-      <c r="M17" s="212"/>
-      <c r="N17" s="215"/>
-      <c r="O17" s="212"/>
-      <c r="P17" s="216"/>
-      <c r="Q17" s="212"/>
-      <c r="R17" s="216"/>
-      <c r="S17" s="218"/>
-      <c r="T17" s="218"/>
-      <c r="U17" s="212"/>
-      <c r="V17" s="215"/>
-      <c r="W17" s="212"/>
-    </row>
-    <row r="18" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="217" t="s">
+      <c r="B17" s="165"/>
+      <c r="C17" s="165"/>
+      <c r="D17" s="165"/>
+      <c r="E17" s="157"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="110"/>
+      <c r="I17" s="160"/>
+      <c r="J17" s="110"/>
+      <c r="K17" s="157"/>
+      <c r="L17" s="110"/>
+      <c r="M17" s="157"/>
+      <c r="N17" s="110"/>
+      <c r="O17" s="157"/>
+      <c r="P17" s="158"/>
+      <c r="Q17" s="157"/>
+      <c r="R17" s="158"/>
+      <c r="S17" s="159"/>
+      <c r="T17" s="159"/>
+      <c r="U17" s="157"/>
+      <c r="V17" s="110"/>
+      <c r="W17" s="157"/>
+    </row>
+    <row r="18" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="113" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="215">
+      <c r="B18" s="110">
         <f>SUM(B9:B17)</f>
         <v>0</v>
       </c>
-      <c r="C18" s="215">
+      <c r="C18" s="110">
         <f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="215">
+      <c r="D18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E18" s="215">
+      <c r="E18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="215">
+      <c r="F18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G18" s="215">
+      <c r="G18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="215">
+      <c r="H18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="215">
+      <c r="I18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="215">
+      <c r="J18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="215">
+      <c r="K18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L18" s="215">
+      <c r="L18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M18" s="215">
+      <c r="M18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N18" s="215">
+      <c r="N18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O18" s="215">
+      <c r="O18" s="110">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P18" s="215">
+      <c r="P18" s="110">
         <f t="shared" ref="P18" si="1">SUM(P9:P17)</f>
         <v>0</v>
       </c>
-      <c r="Q18" s="215">
+      <c r="Q18" s="110">
         <f>SUM(Q9:Q17)</f>
         <v>0</v>
       </c>
-      <c r="R18" s="215">
+      <c r="R18" s="110">
         <f>SUM(R9:R17)</f>
         <v>0</v>
       </c>
-      <c r="S18" s="220">
+      <c r="S18" s="116">
         <f>SUM(S9:S17)</f>
         <v>0</v>
       </c>
-      <c r="T18" s="220">
+      <c r="T18" s="116">
         <f>SUM(T9:T17)</f>
         <v>0</v>
       </c>
-      <c r="U18" s="215">
+      <c r="U18" s="110">
         <f t="shared" ref="U18:W18" si="2">SUM(U9:U17)</f>
         <v>0</v>
       </c>
-      <c r="V18" s="215">
+      <c r="V18" s="110">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="W18" s="215">
+      <c r="W18" s="110">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:23" s="222" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="217"/>
-      <c r="B19" s="215"/>
-      <c r="C19" s="215"/>
-      <c r="D19" s="215"/>
-      <c r="E19" s="215"/>
-      <c r="F19" s="212"/>
-      <c r="G19" s="215"/>
-      <c r="H19" s="215"/>
-      <c r="I19" s="215"/>
-      <c r="J19" s="215"/>
-      <c r="K19" s="215"/>
-      <c r="L19" s="215"/>
-      <c r="M19" s="215"/>
-      <c r="N19" s="215"/>
-      <c r="O19" s="215"/>
-      <c r="P19" s="215"/>
-      <c r="Q19" s="215"/>
-      <c r="R19" s="215"/>
-      <c r="S19" s="220"/>
-      <c r="T19" s="220"/>
-      <c r="U19" s="215"/>
-      <c r="V19" s="215"/>
-      <c r="W19" s="215"/>
-    </row>
-    <row r="20" spans="1:23" s="223" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="113"/>
+      <c r="B19" s="110"/>
+      <c r="C19" s="110"/>
+      <c r="D19" s="110"/>
+      <c r="E19" s="110"/>
+      <c r="F19" s="157"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="110"/>
+      <c r="K19" s="110"/>
+      <c r="L19" s="110"/>
+      <c r="M19" s="110"/>
+      <c r="N19" s="110"/>
+      <c r="O19" s="110"/>
+      <c r="P19" s="110"/>
+      <c r="Q19" s="110"/>
+      <c r="R19" s="110"/>
+      <c r="S19" s="116"/>
+      <c r="T19" s="116"/>
+      <c r="U19" s="110"/>
+      <c r="V19" s="110"/>
+      <c r="W19" s="110"/>
+    </row>
+    <row r="20" spans="1:23" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="113" t="s">
         <v>12</v>
       </c>
@@ -2726,17 +2701,17 @@
     </row>
     <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="2"/>
-      <c r="M22" s="168" t="s">
+      <c r="M22" s="198" t="s">
         <v>48</v>
       </c>
-      <c r="N22" s="168"/>
-      <c r="O22" s="168"/>
-      <c r="P22" s="168"/>
-      <c r="Q22" s="168"/>
-      <c r="R22" s="168"/>
-      <c r="S22" s="168"/>
-      <c r="T22" s="168"/>
-      <c r="U22" s="168"/>
+      <c r="N22" s="198"/>
+      <c r="O22" s="198"/>
+      <c r="P22" s="198"/>
+      <c r="Q22" s="198"/>
+      <c r="R22" s="198"/>
+      <c r="S22" s="198"/>
+      <c r="T22" s="198"/>
+      <c r="U22" s="198"/>
     </row>
     <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D23" s="6"/>
@@ -2745,21 +2720,17 @@
       <c r="M23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N23" s="151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24-06-2026</t>
-        </is>
-      </c>
-      <c r="O23" s="152"/>
-      <c r="P23" s="152"/>
-      <c r="Q23" s="152"/>
-      <c r="R23" s="152"/>
-      <c r="S23" s="153"/>
+      <c r="N23" s="207"/>
+      <c r="O23" s="208"/>
+      <c r="P23" s="208"/>
+      <c r="Q23" s="208"/>
+      <c r="R23" s="208"/>
+      <c r="S23" s="209"/>
       <c r="T23" s="119" t="s">
         <v>38</v>
       </c>
       <c r="U23" s="106">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="W23" s="91" t="s">
         <v>44</v>
@@ -2772,22 +2743,22 @@
       <c r="K24" s="15"/>
       <c r="L24"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="154" t="s">
+      <c r="N24" s="210" t="s">
         <v>49</v>
       </c>
-      <c r="O24" s="155"/>
-      <c r="P24" s="155"/>
-      <c r="Q24" s="155"/>
-      <c r="R24" s="155"/>
-      <c r="S24" s="156"/>
+      <c r="O24" s="211"/>
+      <c r="P24" s="211"/>
+      <c r="Q24" s="211"/>
+      <c r="R24" s="211"/>
+      <c r="S24" s="212"/>
       <c r="T24" s="108" t="s">
         <v>11</v>
       </c>
       <c r="U24" s="107">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="W24" s="118">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
@@ -2799,21 +2770,21 @@
       <c r="E25" s="4"/>
       <c r="J25"/>
       <c r="L25"/>
-      <c r="M25" s="161" t="s">
+      <c r="M25" s="215" t="s">
         <v>16</v>
       </c>
-      <c r="N25" s="162"/>
+      <c r="N25" s="216"/>
       <c r="O25" s="148"/>
       <c r="P25" s="149"/>
       <c r="Q25" s="145">
-        <v>900000</v>
+        <v>180000</v>
       </c>
       <c r="R25" s="146"/>
       <c r="S25" s="147"/>
-      <c r="T25" s="157" t="s">
+      <c r="T25" s="213" t="s">
         <v>17</v>
       </c>
-      <c r="U25" s="158"/>
+      <c r="U25" s="214"/>
       <c r="V25" s="13"/>
       <c r="W25" s="82" t="s">
         <v>45</v>
@@ -2829,11 +2800,11 @@
       <c r="N26" s="80"/>
       <c r="O26" s="126"/>
       <c r="P26" s="127"/>
-      <c r="Q26" s="165">
-        <v>100000</v>
-      </c>
-      <c r="R26" s="166"/>
-      <c r="S26" s="167"/>
+      <c r="Q26" s="188">
+        <v>20000</v>
+      </c>
+      <c r="R26" s="189"/>
+      <c r="S26" s="190"/>
       <c r="T26" s="124"/>
       <c r="U26" s="125"/>
       <c r="V26" s="13"/>
@@ -2851,20 +2822,18 @@
         <v>18</v>
       </c>
       <c r="N27" s="80"/>
-      <c r="O27" s="163"/>
-      <c r="P27" s="169"/>
-      <c r="Q27" s="165" t="s">
-        <v>64</v>
-      </c>
-      <c r="R27" s="166"/>
-      <c r="S27" s="167"/>
-      <c r="T27" s="176" t="s">
+      <c r="O27" s="186"/>
+      <c r="P27" s="187"/>
+      <c r="Q27" s="188"/>
+      <c r="R27" s="189"/>
+      <c r="S27" s="190"/>
+      <c r="T27" s="205" t="s">
         <v>19</v>
       </c>
-      <c r="U27" s="177"/>
+      <c r="U27" s="206"/>
       <c r="V27" s="19"/>
       <c r="W27" s="92">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
@@ -2877,19 +2846,19 @@
         <v>0</v>
       </c>
       <c r="L28"/>
-      <c r="M28" s="174" t="s">
+      <c r="M28" s="203" t="s">
         <v>20</v>
       </c>
-      <c r="N28" s="175"/>
-      <c r="O28" s="163"/>
-      <c r="P28" s="169"/>
-      <c r="Q28" s="165"/>
-      <c r="R28" s="166"/>
-      <c r="S28" s="167"/>
-      <c r="T28" s="172" t="s">
+      <c r="N28" s="204"/>
+      <c r="O28" s="186"/>
+      <c r="P28" s="187"/>
+      <c r="Q28" s="188"/>
+      <c r="R28" s="189"/>
+      <c r="S28" s="190"/>
+      <c r="T28" s="201" t="s">
         <v>39</v>
       </c>
-      <c r="U28" s="173"/>
+      <c r="U28" s="202"/>
       <c r="V28" s="21"/>
       <c r="W28" s="13"/>
     </row>
@@ -2904,19 +2873,19 @@
       </c>
       <c r="K29" s="24"/>
       <c r="L29"/>
-      <c r="M29" s="174" t="s">
+      <c r="M29" s="203" t="s">
         <v>21</v>
       </c>
-      <c r="N29" s="175"/>
-      <c r="O29" s="163"/>
-      <c r="P29" s="169"/>
-      <c r="Q29" s="165"/>
-      <c r="R29" s="166"/>
-      <c r="S29" s="167"/>
-      <c r="T29" s="170" t="s">
+      <c r="N29" s="204"/>
+      <c r="O29" s="186"/>
+      <c r="P29" s="187"/>
+      <c r="Q29" s="188"/>
+      <c r="R29" s="189"/>
+      <c r="S29" s="190"/>
+      <c r="T29" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="U29" s="171"/>
+      <c r="U29" s="200"/>
       <c r="W29" s="93" t="str">
         <f>U23</f>
       </c>
@@ -2932,19 +2901,19 @@
         <v>0</v>
       </c>
       <c r="L30"/>
-      <c r="M30" s="174" t="s">
+      <c r="M30" s="203" t="s">
         <v>22</v>
       </c>
-      <c r="N30" s="175"/>
-      <c r="O30" s="163"/>
-      <c r="P30" s="164"/>
-      <c r="Q30" s="165"/>
-      <c r="R30" s="166"/>
-      <c r="S30" s="167"/>
-      <c r="T30" s="178" t="s">
+      <c r="N30" s="204"/>
+      <c r="O30" s="186"/>
+      <c r="P30" s="217"/>
+      <c r="Q30" s="188"/>
+      <c r="R30" s="189"/>
+      <c r="S30" s="190"/>
+      <c r="T30" s="218" t="s">
         <v>41</v>
       </c>
-      <c r="U30" s="179"/>
+      <c r="U30" s="219"/>
       <c r="V30" s="24"/>
       <c r="W30" s="21" t="str">
         <f>Q34</f>
@@ -2961,15 +2930,15 @@
         <v>0</v>
       </c>
       <c r="L31"/>
-      <c r="M31" s="174" t="s">
+      <c r="M31" s="203" t="s">
         <v>23</v>
       </c>
-      <c r="N31" s="175"/>
-      <c r="O31" s="163"/>
-      <c r="P31" s="169"/>
-      <c r="Q31" s="165"/>
-      <c r="R31" s="166"/>
-      <c r="S31" s="167"/>
+      <c r="N31" s="204"/>
+      <c r="O31" s="186"/>
+      <c r="P31" s="187"/>
+      <c r="Q31" s="188"/>
+      <c r="R31" s="189"/>
+      <c r="S31" s="190"/>
       <c r="T31" s="28"/>
       <c r="U31" s="26"/>
     </row>
@@ -2984,15 +2953,15 @@
         <v>0</v>
       </c>
       <c r="L32"/>
-      <c r="M32" s="174" t="s">
+      <c r="M32" s="203" t="s">
         <v>24</v>
       </c>
-      <c r="N32" s="175"/>
-      <c r="O32" s="163"/>
-      <c r="P32" s="169"/>
-      <c r="Q32" s="165"/>
-      <c r="R32" s="166"/>
-      <c r="S32" s="167"/>
+      <c r="N32" s="204"/>
+      <c r="O32" s="186"/>
+      <c r="P32" s="187"/>
+      <c r="Q32" s="188"/>
+      <c r="R32" s="189"/>
+      <c r="S32" s="190"/>
       <c r="T32" s="28"/>
       <c r="U32" s="26"/>
       <c r="W32" s="82" t="s">
@@ -3014,11 +2983,11 @@
         <v>25</v>
       </c>
       <c r="N33" s="81"/>
-      <c r="O33" s="163"/>
-      <c r="P33" s="169"/>
-      <c r="Q33" s="165"/>
-      <c r="R33" s="166"/>
-      <c r="S33" s="167"/>
+      <c r="O33" s="186"/>
+      <c r="P33" s="187"/>
+      <c r="Q33" s="188"/>
+      <c r="R33" s="189"/>
+      <c r="S33" s="190"/>
       <c r="T33" s="28"/>
       <c r="U33" s="26"/>
       <c r="W33" s="117" t="e">
@@ -3037,17 +3006,17 @@
         <v>0</v>
       </c>
       <c r="L34" s="8"/>
-      <c r="M34" s="183" t="s">
+      <c r="M34" s="191" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="184"/>
-      <c r="O34" s="185"/>
-      <c r="P34" s="186"/>
-      <c r="Q34" s="165">
-        <v>2000000</v>
-      </c>
-      <c r="R34" s="166"/>
-      <c r="S34" s="167"/>
+      <c r="N34" s="192"/>
+      <c r="O34" s="193"/>
+      <c r="P34" s="194"/>
+      <c r="Q34" s="188">
+        <v>1000000</v>
+      </c>
+      <c r="R34" s="189"/>
+      <c r="S34" s="190"/>
       <c r="T34" s="30"/>
       <c r="U34" s="29"/>
       <c r="V34" s="1"/>
@@ -3065,23 +3034,23 @@
         <v>0</v>
       </c>
       <c r="L35"/>
-      <c r="M35" s="193" t="s">
+      <c r="M35" s="195" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="194"/>
-      <c r="O35" s="195"/>
-      <c r="P35" s="181" t="s">
+      <c r="N35" s="196"/>
+      <c r="O35" s="197"/>
+      <c r="P35" s="167" t="s">
         <v>28</v>
       </c>
-      <c r="Q35" s="182"/>
-      <c r="R35" s="181" t="s">
+      <c r="Q35" s="169"/>
+      <c r="R35" s="167" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="182"/>
-      <c r="T35" s="181" t="s">
+      <c r="S35" s="169"/>
+      <c r="T35" s="167" t="s">
         <v>30</v>
       </c>
-      <c r="U35" s="182"/>
+      <c r="U35" s="169"/>
       <c r="V35" s="1"/>
       <c r="W35" s="1"/>
     </row>
@@ -3138,169 +3107,131 @@
       </c>
       <c r="K37" s="24"/>
       <c r="L37"/>
-      <c r="M37" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">01-01-2026</t>
-        </is>
-      </c>
-      <c r="N37" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SANTANDER</t>
-        </is>
-      </c>
-      <c r="O37" s="39">
-        <v>100000</v>
-      </c>
-      <c r="P37" s="205"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="38"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="151"/>
       <c r="Q37" s="77"/>
-      <c r="R37" s="207"/>
+      <c r="R37" s="153"/>
       <c r="S37" s="78"/>
-      <c r="T37" s="206"/>
+      <c r="T37" s="152"/>
       <c r="U37" s="74"/>
       <c r="V37" s="1"/>
       <c r="W37" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A38" s="1"/>
+    <row r="38" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="20"/>
+      <c r="C38" s="32"/>
       <c r="I38" s="41">
-        <f>
-          L
-          <row r="37" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-            <c r="A37" s="1"/>
-            <c r="I37" s="41">
-              <f>L$1</f>
-              <v>0</v>
-            </c>
-            <c r="J37" s="27">
-              <f>L9</f>
-              <v>0</v>
-            </c>
-            <c r="K37" s="24"/>
-            <c r="L37"/>
-            <c r="M37" s="37" t="inlineStr">
-              <is>
-                <t xml:space="preserve">01-01-2026</t>
-              </is>
-            </c>
-            <c r="N37" s="38" t="inlineStr">
-              <is>
-                <t xml:space="preserve">SANTANDER</t>
-              </is>
-            </c>
-            <c r="O37" s="39">
-              <v>100000</v>
-            </c>
-            <c r="P37" s="205"/>
-            <c r="Q37" s="77"/>
-            <c r="R37" s="207"/>
-            <c r="S37" s="78"/>
-            <c r="T37" s="206"/>
-            <c r="U37" s="74"/>
-            <c r="V37" s="1"/>
-            <c r="W37" s="18" t="s">
-              <v>14</v>
-            </c>
-          </row>
-        </f>
+        <f t="shared" ref="I38:I45" si="6">L$1</f>
         <v>0</v>
       </c>
       <c r="J38" s="27">
-        <f>L9</f>
-        <v>0</v>
-      </c>
-      <c r="K38" s="24"/>
-      <c r="L38"/>
-      <c r="M38" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">01-01-2026</t>
-        </is>
-      </c>
-      <c r="N38" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SANTANDER</t>
-        </is>
-      </c>
-      <c r="O38" s="39">
-        <v>100000</v>
-      </c>
-      <c r="P38" s="205"/>
-      <c r="Q38" s="77"/>
-      <c r="R38" s="207"/>
-      <c r="S38" s="78"/>
-      <c r="T38" s="206"/>
-      <c r="U38" s="74"/>
+        <f t="shared" ref="J38:J45" si="7">L10</f>
+        <v>0</v>
+      </c>
+      <c r="L38" s="105"/>
+      <c r="M38" s="171" t="s">
+        <v>42</v>
+      </c>
+      <c r="N38" s="179"/>
+      <c r="O38" s="150"/>
+      <c r="P38" s="152"/>
+      <c r="Q38" s="75"/>
+      <c r="R38" s="154"/>
+      <c r="S38" s="73"/>
+      <c r="T38" s="152"/>
+      <c r="U38" s="76"/>
       <c r="V38" s="1"/>
-      <c r="W38" s="18"/>
-    </row>
-    <row r="39" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W38" s="1"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B39" s="20"/>
       <c r="C39" s="32"/>
       <c r="I39" s="41">
-        <f t="shared" ref="I39:I46" si="6">L$1</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="J39" s="27">
-        <f t="shared" ref="J39:J46" si="7">L10</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="K39" s="24"/>
       <c r="L39" s="105"/>
-      <c r="M39" s="159" t="s">
-        <v>42</v>
-      </c>
-      <c r="N39" s="160"/>
-      <c r="O39" s="150">
-        <f>SUMA(O37:O38)</f>
-      </c>
-      <c r="P39" s="206"/>
-      <c r="Q39" s="75"/>
-      <c r="R39" s="208"/>
+      <c r="M39" s="37"/>
+      <c r="N39" s="38"/>
+      <c r="O39" s="39"/>
+      <c r="P39" s="152"/>
+      <c r="Q39" s="68"/>
+      <c r="R39" s="154"/>
       <c r="S39" s="73"/>
-      <c r="T39" s="206"/>
-      <c r="U39" s="76"/>
+      <c r="T39" s="152"/>
+      <c r="U39" s="68"/>
       <c r="V39" s="1"/>
       <c r="W39" s="1"/>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="O40" s="0"/>
-      <c r="N40" s="0"/>
-      <c r="M40" s="0"/>
+    <row r="40" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B40" s="20"/>
       <c r="C40" s="32"/>
+      <c r="D40" s="44"/>
+      <c r="E40" s="43"/>
       <c r="I40" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="J40" s="27">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="K40" s="24"/>
+      <c r="L40" s="105"/>
+      <c r="M40" s="37"/>
+      <c r="N40" s="38"/>
+      <c r="O40" s="39"/>
+      <c r="P40" s="152"/>
+      <c r="Q40" s="66"/>
+      <c r="R40" s="154"/>
+      <c r="S40" s="74"/>
+      <c r="T40" s="152"/>
+      <c r="U40" s="68"/>
+      <c r="V40" s="1"/>
+      <c r="W40" s="1"/>
+    </row>
+    <row r="41" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="20"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="I41" s="41">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
       <c r="J41" s="27">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K41" s="24"/>
       <c r="L41" s="105"/>
-      <c r="M41" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="N41" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="O41" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="P41" s="206"/>
-      <c r="Q41" s="68"/>
-      <c r="R41" s="208"/>
-      <c r="S41" s="73"/>
-      <c r="T41" s="206"/>
+      <c r="M41" s="37"/>
+      <c r="N41" s="38"/>
+      <c r="O41" s="39"/>
+      <c r="P41" s="152"/>
+      <c r="Q41" s="66"/>
+      <c r="R41" s="154"/>
+      <c r="S41" s="74"/>
+      <c r="T41" s="152"/>
       <c r="U41" s="68"/>
       <c r="V41" s="1"/>
       <c r="W41" s="1"/>
     </row>
-    <row r="41" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B42" s="20"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="43"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="47"/>
       <c r="I42" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -3309,25 +3240,27 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="K42" s="24"/>
       <c r="L42" s="105"/>
       <c r="M42" s="37"/>
       <c r="N42" s="38"/>
       <c r="O42" s="39"/>
-      <c r="P42" s="206"/>
+      <c r="P42" s="152"/>
       <c r="Q42" s="66"/>
-      <c r="R42" s="208"/>
-      <c r="S42" s="74"/>
-      <c r="T42" s="206"/>
+      <c r="R42" s="154"/>
+      <c r="S42" s="73"/>
+      <c r="T42" s="152"/>
       <c r="U42" s="68"/>
       <c r="V42" s="1"/>
       <c r="W42" s="1"/>
     </row>
-    <row r="42" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A43" s="104"/>
       <c r="B43" s="20"/>
       <c r="C43" s="32"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
+      <c r="D43" s="170"/>
+      <c r="E43" s="170"/>
+      <c r="F43" s="47"/>
+      <c r="G43" s="8"/>
       <c r="I43" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -3341,21 +3274,21 @@
       <c r="M43" s="37"/>
       <c r="N43" s="38"/>
       <c r="O43" s="39"/>
-      <c r="P43" s="206"/>
+      <c r="P43" s="152"/>
       <c r="Q43" s="66"/>
-      <c r="R43" s="208"/>
-      <c r="S43" s="74"/>
-      <c r="T43" s="206"/>
+      <c r="R43" s="152"/>
+      <c r="S43" s="67"/>
+      <c r="T43" s="152"/>
       <c r="U43" s="68"/>
-      <c r="V43" s="1"/>
-      <c r="W43" s="1"/>
-    </row>
-    <row r="43" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.6">
+    </row>
+    <row r="44" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="25"/>
       <c r="B44" s="20"/>
       <c r="C44" s="25"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="23"/>
-      <c r="F44" s="47"/>
+      <c r="D44" s="170"/>
+      <c r="E44" s="170"/>
+      <c r="F44" s="48"/>
+      <c r="H44" s="64"/>
       <c r="I44" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -3364,27 +3297,26 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="K44" s="24"/>
       <c r="L44" s="105"/>
       <c r="M44" s="37"/>
       <c r="N44" s="38"/>
       <c r="O44" s="39"/>
-      <c r="P44" s="206"/>
+      <c r="P44" s="152"/>
       <c r="Q44" s="66"/>
-      <c r="R44" s="208"/>
-      <c r="S44" s="73"/>
-      <c r="T44" s="206"/>
+      <c r="R44" s="152"/>
+      <c r="S44" s="67"/>
+      <c r="T44" s="152"/>
       <c r="U44" s="68"/>
-      <c r="V44" s="1"/>
-      <c r="W44" s="1"/>
-    </row>
-    <row r="44" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A45" s="104"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="180"/>
-      <c r="E45" s="180"/>
-      <c r="F45" s="47"/>
-      <c r="G45" s="8"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A45" s="25"/>
+      <c r="B45" s="25"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="170"/>
+      <c r="E45" s="170"/>
+      <c r="F45" s="23"/>
+      <c r="H45" s="64"/>
       <c r="I45" s="41">
         <f t="shared" si="6"/>
         <v>0</v>
@@ -3393,148 +3325,114 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="K45" s="24"/>
       <c r="L45" s="105"/>
       <c r="M45" s="37"/>
       <c r="N45" s="38"/>
       <c r="O45" s="39"/>
-      <c r="P45" s="206"/>
+      <c r="P45" s="152"/>
       <c r="Q45" s="66"/>
-      <c r="R45" s="206"/>
-      <c r="S45" s="67"/>
-      <c r="T45" s="206"/>
+      <c r="R45" s="152"/>
+      <c r="S45" s="72"/>
+      <c r="T45" s="152"/>
       <c r="U45" s="68"/>
     </row>
-    <row r="45" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="25"/>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A46" s="20"/>
       <c r="B46" s="20"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="180"/>
-      <c r="E46" s="180"/>
-      <c r="F46" s="48"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="170"/>
+      <c r="E46" s="170"/>
+      <c r="F46" s="49"/>
       <c r="H46" s="64"/>
-      <c r="I46" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J46" s="27">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="K46" s="24"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="53">
+        <f>SUM(J28:J45)</f>
+        <v>0</v>
+      </c>
       <c r="L46" s="105"/>
       <c r="M46" s="37"/>
       <c r="N46" s="38"/>
       <c r="O46" s="39"/>
-      <c r="P46" s="206"/>
+      <c r="P46" s="152"/>
       <c r="Q46" s="66"/>
-      <c r="R46" s="206"/>
+      <c r="R46" s="152"/>
       <c r="S46" s="67"/>
-      <c r="T46" s="206"/>
+      <c r="T46" s="152"/>
       <c r="U46" s="68"/>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A47" s="25"/>
-      <c r="B47" s="25"/>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
       <c r="C47" s="40"/>
-      <c r="D47" s="180"/>
-      <c r="E47" s="180"/>
-      <c r="F47" s="23"/>
+      <c r="D47" s="170"/>
+      <c r="E47" s="170"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="1"/>
       <c r="H47" s="64"/>
-      <c r="I47" s="41">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J47" s="27">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
+      <c r="I47" s="13"/>
+      <c r="J47" s="53"/>
+      <c r="K47" s="24"/>
       <c r="L47" s="105"/>
       <c r="M47" s="37"/>
       <c r="N47" s="38"/>
       <c r="O47" s="39"/>
-      <c r="P47" s="206"/>
+      <c r="P47" s="152"/>
       <c r="Q47" s="66"/>
-      <c r="R47" s="206"/>
-      <c r="S47" s="72"/>
-      <c r="T47" s="206"/>
-      <c r="U47" s="68"/>
-    </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="40"/>
-      <c r="D48" s="180"/>
-      <c r="E48" s="180"/>
-      <c r="F48" s="49"/>
-      <c r="H48" s="64"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="53">
-        <f>SUM(J28:J46)</f>
-        <v>0</v>
-      </c>
-      <c r="L47" s="105"/>
-      <c r="M47" s="37"/>
-      <c r="N47" s="38"/>
-      <c r="O47" s="39"/>
-      <c r="P47" s="206"/>
-      <c r="Q47" s="66"/>
-      <c r="R47" s="206"/>
+      <c r="R47" s="152"/>
       <c r="S47" s="67"/>
-      <c r="T47" s="206"/>
+      <c r="T47" s="152"/>
       <c r="U47" s="68"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" s="20"/>
       <c r="B48" s="20"/>
       <c r="C48" s="40"/>
-      <c r="D48" s="180"/>
-      <c r="E48" s="180"/>
-      <c r="F48" s="17"/>
+      <c r="D48" s="170"/>
+      <c r="E48" s="170"/>
+      <c r="F48" s="23"/>
       <c r="G48" s="1"/>
       <c r="H48" s="64"/>
       <c r="I48" s="13"/>
       <c r="J48" s="53"/>
-      <c r="K48" s="24"/>
       <c r="L48" s="105"/>
       <c r="M48" s="37"/>
       <c r="N48" s="38"/>
       <c r="O48" s="39"/>
-      <c r="P48" s="206"/>
+      <c r="P48" s="152"/>
       <c r="Q48" s="66"/>
-      <c r="R48" s="206"/>
+      <c r="R48" s="152"/>
       <c r="S48" s="67"/>
-      <c r="T48" s="206"/>
+      <c r="T48" s="154"/>
       <c r="U48" s="68"/>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="40"/>
-      <c r="D49" s="180"/>
-      <c r="E49" s="180"/>
+      <c r="D49" s="170"/>
+      <c r="E49" s="170"/>
       <c r="F49" s="23"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="64"/>
+      <c r="H49" s="46"/>
       <c r="I49" s="13"/>
       <c r="J49" s="53"/>
       <c r="L49" s="105"/>
       <c r="M49" s="37"/>
       <c r="N49" s="38"/>
       <c r="O49" s="39"/>
-      <c r="P49" s="206"/>
+      <c r="P49" s="152"/>
       <c r="Q49" s="66"/>
-      <c r="R49" s="206"/>
+      <c r="R49" s="152"/>
       <c r="S49" s="67"/>
-      <c r="T49" s="208"/>
+      <c r="T49" s="154"/>
       <c r="U49" s="68"/>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" s="20"/>
       <c r="B50" s="20"/>
       <c r="C50" s="40"/>
-      <c r="D50" s="180"/>
-      <c r="E50" s="180"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="25"/>
       <c r="F50" s="23"/>
       <c r="G50" s="1"/>
       <c r="H50" s="46"/>
@@ -3544,19 +3442,19 @@
       <c r="M50" s="37"/>
       <c r="N50" s="38"/>
       <c r="O50" s="39"/>
-      <c r="P50" s="206"/>
+      <c r="P50" s="152"/>
       <c r="Q50" s="66"/>
-      <c r="R50" s="206"/>
+      <c r="R50" s="152"/>
       <c r="S50" s="67"/>
-      <c r="T50" s="208"/>
+      <c r="T50" s="154"/>
       <c r="U50" s="68"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" s="20"/>
       <c r="B51" s="20"/>
       <c r="C51" s="40"/>
-      <c r="D51" s="23"/>
-      <c r="E51" s="25"/>
+      <c r="D51" s="185"/>
+      <c r="E51" s="185"/>
       <c r="F51" s="23"/>
       <c r="G51" s="1"/>
       <c r="H51" s="46"/>
@@ -3566,63 +3464,63 @@
       <c r="M51" s="37"/>
       <c r="N51" s="38"/>
       <c r="O51" s="39"/>
-      <c r="P51" s="206"/>
+      <c r="P51" s="151"/>
       <c r="Q51" s="66"/>
-      <c r="R51" s="206"/>
+      <c r="R51" s="152"/>
       <c r="S51" s="67"/>
-      <c r="T51" s="208"/>
+      <c r="T51" s="154"/>
       <c r="U51" s="68"/>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A52" s="20"/>
-      <c r="B52" s="20"/>
+      <c r="B52" s="51"/>
       <c r="C52" s="40"/>
-      <c r="D52" s="190"/>
-      <c r="E52" s="190"/>
+      <c r="D52" s="178"/>
+      <c r="E52" s="178"/>
       <c r="F52" s="23"/>
       <c r="G52" s="1"/>
       <c r="H52" s="46"/>
-      <c r="I52" s="13"/>
+      <c r="I52" s="50"/>
       <c r="J52" s="53"/>
       <c r="L52" s="105"/>
       <c r="M52" s="37"/>
       <c r="N52" s="38"/>
       <c r="O52" s="39"/>
-      <c r="P52" s="205"/>
+      <c r="P52" s="151"/>
       <c r="Q52" s="66"/>
-      <c r="R52" s="206"/>
+      <c r="R52" s="152"/>
       <c r="S52" s="67"/>
-      <c r="T52" s="208"/>
+      <c r="T52" s="154"/>
       <c r="U52" s="68"/>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A53" s="20"/>
+      <c r="A53" s="25"/>
       <c r="B53" s="51"/>
       <c r="C53" s="40"/>
-      <c r="D53" s="202"/>
-      <c r="E53" s="202"/>
+      <c r="D53" s="166"/>
+      <c r="E53" s="166"/>
       <c r="F53" s="23"/>
       <c r="G53" s="1"/>
       <c r="H53" s="46"/>
       <c r="I53" s="50"/>
       <c r="J53" s="53"/>
-      <c r="L53" s="105"/>
+      <c r="L53" s="18"/>
       <c r="M53" s="37"/>
       <c r="N53" s="38"/>
       <c r="O53" s="39"/>
-      <c r="P53" s="205"/>
+      <c r="P53" s="152"/>
       <c r="Q53" s="66"/>
-      <c r="R53" s="206"/>
+      <c r="R53" s="152"/>
       <c r="S53" s="67"/>
-      <c r="T53" s="208"/>
+      <c r="T53" s="154"/>
       <c r="U53" s="68"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A54" s="25"/>
+      <c r="A54" s="20"/>
       <c r="B54" s="51"/>
       <c r="C54" s="40"/>
-      <c r="D54" s="189"/>
-      <c r="E54" s="189"/>
+      <c r="D54" s="166"/>
+      <c r="E54" s="166"/>
       <c r="F54" s="23"/>
       <c r="G54" s="1"/>
       <c r="H54" s="46"/>
@@ -3632,19 +3530,19 @@
       <c r="M54" s="37"/>
       <c r="N54" s="38"/>
       <c r="O54" s="39"/>
-      <c r="P54" s="206"/>
+      <c r="P54" s="152"/>
       <c r="Q54" s="66"/>
-      <c r="R54" s="206"/>
+      <c r="R54" s="152"/>
       <c r="S54" s="67"/>
-      <c r="T54" s="208"/>
+      <c r="T54" s="154"/>
       <c r="U54" s="68"/>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A55" s="20"/>
       <c r="B55" s="51"/>
       <c r="C55" s="40"/>
-      <c r="D55" s="189"/>
-      <c r="E55" s="189"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
       <c r="F55" s="23"/>
       <c r="G55" s="1"/>
       <c r="H55" s="46"/>
@@ -3654,16 +3552,16 @@
       <c r="M55" s="37"/>
       <c r="N55" s="38"/>
       <c r="O55" s="39"/>
-      <c r="P55" s="206"/>
+      <c r="P55" s="152"/>
       <c r="Q55" s="66"/>
-      <c r="R55" s="206"/>
+      <c r="R55" s="152"/>
       <c r="S55" s="67"/>
-      <c r="T55" s="208"/>
+      <c r="T55" s="154"/>
       <c r="U55" s="68"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" s="20"/>
-      <c r="B56" s="51"/>
+      <c r="B56"/>
       <c r="C56" s="40"/>
       <c r="D56" s="22"/>
       <c r="E56" s="22"/>
@@ -3676,11 +3574,11 @@
       <c r="M56" s="37"/>
       <c r="N56" s="38"/>
       <c r="O56" s="39"/>
-      <c r="P56" s="206"/>
+      <c r="P56" s="152"/>
       <c r="Q56" s="66"/>
-      <c r="R56" s="206"/>
+      <c r="R56" s="152"/>
       <c r="S56" s="67"/>
-      <c r="T56" s="208"/>
+      <c r="T56" s="154"/>
       <c r="U56" s="68"/>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.3">
@@ -3698,11 +3596,11 @@
       <c r="M57" s="37"/>
       <c r="N57" s="38"/>
       <c r="O57" s="39"/>
-      <c r="P57" s="206"/>
+      <c r="P57" s="152"/>
       <c r="Q57" s="66"/>
-      <c r="R57" s="206"/>
+      <c r="R57" s="152"/>
       <c r="S57" s="67"/>
-      <c r="T57" s="208"/>
+      <c r="T57" s="154"/>
       <c r="U57" s="68"/>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.3">
@@ -3720,11 +3618,11 @@
       <c r="M58" s="37"/>
       <c r="N58" s="38"/>
       <c r="O58" s="39"/>
-      <c r="P58" s="206"/>
+      <c r="P58" s="152"/>
       <c r="Q58" s="66"/>
-      <c r="R58" s="206"/>
+      <c r="R58" s="152"/>
       <c r="S58" s="67"/>
-      <c r="T58" s="208"/>
+      <c r="T58" s="154"/>
       <c r="U58" s="68"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.3">
@@ -3742,19 +3640,19 @@
       <c r="M59" s="37"/>
       <c r="N59" s="38"/>
       <c r="O59" s="39"/>
-      <c r="P59" s="206"/>
+      <c r="P59" s="152"/>
       <c r="Q59" s="66"/>
-      <c r="R59" s="206"/>
+      <c r="R59" s="152"/>
       <c r="S59" s="67"/>
-      <c r="T59" s="208"/>
+      <c r="T59" s="154"/>
       <c r="U59" s="68"/>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A60" s="20"/>
+      <c r="A60" s="25"/>
       <c r="B60"/>
       <c r="C60" s="40"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
+      <c r="D60" s="166"/>
+      <c r="E60" s="166"/>
       <c r="F60" s="23"/>
       <c r="G60" s="1"/>
       <c r="H60" s="46"/>
@@ -3764,19 +3662,19 @@
       <c r="M60" s="37"/>
       <c r="N60" s="38"/>
       <c r="O60" s="39"/>
-      <c r="P60" s="206"/>
+      <c r="P60" s="152"/>
       <c r="Q60" s="66"/>
-      <c r="R60" s="206"/>
+      <c r="R60" s="152"/>
       <c r="S60" s="67"/>
-      <c r="T60" s="208"/>
+      <c r="T60" s="154"/>
       <c r="U60" s="68"/>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A61" s="25"/>
       <c r="B61"/>
       <c r="C61" s="40"/>
-      <c r="D61" s="189"/>
-      <c r="E61" s="189"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
       <c r="F61" s="23"/>
       <c r="G61" s="1"/>
       <c r="H61" s="46"/>
@@ -3786,11 +3684,11 @@
       <c r="M61" s="37"/>
       <c r="N61" s="38"/>
       <c r="O61" s="39"/>
-      <c r="P61" s="206"/>
-      <c r="Q61" s="66"/>
-      <c r="R61" s="206"/>
-      <c r="S61" s="67"/>
-      <c r="T61" s="208"/>
+      <c r="P61" s="152"/>
+      <c r="Q61" s="135"/>
+      <c r="R61" s="155"/>
+      <c r="S61" s="88"/>
+      <c r="T61" s="154"/>
       <c r="U61" s="68"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.3">
@@ -3808,11 +3706,11 @@
       <c r="M62" s="37"/>
       <c r="N62" s="38"/>
       <c r="O62" s="39"/>
-      <c r="P62" s="206"/>
+      <c r="P62" s="152"/>
       <c r="Q62" s="135"/>
-      <c r="R62" s="209"/>
+      <c r="R62" s="155"/>
       <c r="S62" s="88"/>
-      <c r="T62" s="208"/>
+      <c r="T62" s="154"/>
       <c r="U62" s="68"/>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.3">
@@ -3830,19 +3728,19 @@
       <c r="M63" s="37"/>
       <c r="N63" s="38"/>
       <c r="O63" s="39"/>
-      <c r="P63" s="206"/>
+      <c r="P63" s="152"/>
       <c r="Q63" s="135"/>
-      <c r="R63" s="209"/>
+      <c r="R63" s="155"/>
       <c r="S63" s="88"/>
-      <c r="T63" s="208"/>
+      <c r="T63" s="154"/>
       <c r="U63" s="68"/>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="25"/>
       <c r="B64"/>
       <c r="C64" s="40"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
+      <c r="D64" s="166"/>
+      <c r="E64" s="166"/>
       <c r="F64" s="23"/>
       <c r="G64" s="1"/>
       <c r="H64" s="46"/>
@@ -3852,403 +3750,342 @@
       <c r="M64" s="37"/>
       <c r="N64" s="38"/>
       <c r="O64" s="39"/>
-      <c r="P64" s="206"/>
-      <c r="Q64" s="135"/>
-      <c r="R64" s="209"/>
+      <c r="P64" s="152"/>
+      <c r="Q64" s="84"/>
+      <c r="R64" s="155"/>
       <c r="S64" s="88"/>
-      <c r="T64" s="208"/>
-      <c r="U64" s="68"/>
-    </row>
-    <row r="65" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="T64" s="154"/>
+      <c r="U64" s="71"/>
+    </row>
+    <row r="65" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="25"/>
       <c r="B65"/>
       <c r="C65" s="40"/>
-      <c r="D65" s="189"/>
-      <c r="E65" s="189"/>
-      <c r="F65" s="23"/>
+      <c r="D65" s="166"/>
+      <c r="E65" s="166"/>
+      <c r="F65" s="20"/>
       <c r="G65" s="1"/>
       <c r="H65" s="46"/>
       <c r="I65" s="50"/>
       <c r="J65" s="53"/>
-      <c r="L65" s="18"/>
-      <c r="M65" s="37"/>
-      <c r="N65" s="38"/>
-      <c r="O65" s="39"/>
-      <c r="P65" s="206"/>
-      <c r="Q65" s="84"/>
-      <c r="R65" s="209"/>
-      <c r="S65" s="88"/>
-      <c r="T65" s="208"/>
-      <c r="U65" s="71"/>
-    </row>
-    <row r="66" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L65"/>
+      <c r="M65" s="171" t="s">
+        <v>34</v>
+      </c>
+      <c r="N65" s="172"/>
+      <c r="O65" s="42"/>
+      <c r="P65" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q65" s="42"/>
+      <c r="R65" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="S65" s="42"/>
+      <c r="T65" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="U65" s="42"/>
+    </row>
+    <row r="66" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="25"/>
       <c r="B66"/>
-      <c r="C66" s="40"/>
-      <c r="D66" s="189"/>
-      <c r="E66" s="189"/>
-      <c r="F66" s="20"/>
+      <c r="C66" s="90"/>
+      <c r="D66" s="166"/>
+      <c r="E66" s="166"/>
+      <c r="F66" s="23"/>
       <c r="G66" s="1"/>
       <c r="H66" s="46"/>
       <c r="I66" s="50"/>
-      <c r="J66" s="53"/>
+      <c r="J66"/>
       <c r="L66"/>
-      <c r="M66" s="159" t="s">
-        <v>34</v>
-      </c>
-      <c r="N66" s="196"/>
-      <c r="O66" s="42"/>
-      <c r="P66" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q66" s="42">
-        <f>SUMA(Q37:Q38)</f>
-      </c>
-      <c r="R66" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="S66" s="42">
-        <f>SUMA(S37:S38)</f>
-      </c>
-      <c r="T66" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="U66" s="42">
-        <f>SUMA(U37:U38)</f>
-      </c>
-    </row>
-    <row r="67" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M66" s="54"/>
+      <c r="N66" s="55"/>
+      <c r="O66" s="70"/>
+      <c r="P66" s="23"/>
+      <c r="Q66" s="69"/>
+      <c r="R66" s="70"/>
+      <c r="S66" s="70"/>
+      <c r="T66" s="6"/>
+    </row>
+    <row r="67" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="25"/>
       <c r="B67"/>
-      <c r="C67" s="90"/>
-      <c r="D67" s="189"/>
-      <c r="E67" s="189"/>
+      <c r="C67" s="25"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
       <c r="F67" s="23"/>
       <c r="G67" s="1"/>
       <c r="H67" s="46"/>
       <c r="I67" s="50"/>
       <c r="J67"/>
       <c r="L67"/>
-      <c r="M67" s="54"/>
-      <c r="N67" s="55"/>
-      <c r="O67" s="70"/>
-      <c r="P67" s="23"/>
-      <c r="Q67" s="69"/>
-      <c r="R67" s="70"/>
-      <c r="S67" s="70"/>
-      <c r="T67" s="6"/>
-    </row>
-    <row r="68" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M67" s="167" t="s">
+        <v>47</v>
+      </c>
+      <c r="N67" s="168"/>
+      <c r="O67" s="169"/>
+      <c r="P67" s="181"/>
+      <c r="Q67" s="182"/>
+      <c r="R67" s="167" t="s">
+        <v>37</v>
+      </c>
+      <c r="S67" s="168"/>
+      <c r="T67" s="183" t="str">
+        <f>Q25</f>
+      </c>
+      <c r="U67" s="184"/>
+    </row>
+    <row r="68" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="25"/>
       <c r="B68"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="23"/>
+      <c r="D68" s="166"/>
+      <c r="E68" s="166"/>
+      <c r="F68" s="63"/>
       <c r="G68" s="1"/>
       <c r="H68" s="46"/>
       <c r="I68" s="50"/>
       <c r="J68"/>
       <c r="L68"/>
-      <c r="M68" s="181" t="s">
-        <v>47</v>
-      </c>
-      <c r="N68" s="204"/>
-      <c r="O68" s="182"/>
-      <c r="P68" s="191"/>
-      <c r="Q68" s="192"/>
-      <c r="R68" s="181" t="s">
-        <v>37</v>
-      </c>
-      <c r="S68" s="204"/>
-      <c r="T68" s="187" t="str">
-        <f>Q25</f>
-      </c>
-      <c r="U68" s="188"/>
+      <c r="M68" s="56"/>
+      <c r="N68" s="83"/>
+      <c r="O68" s="83"/>
+      <c r="P68" s="57"/>
+      <c r="Q68" s="58"/>
+      <c r="R68" s="58"/>
+      <c r="S68" s="58"/>
+      <c r="T68" s="56"/>
+      <c r="U68" s="56"/>
     </row>
     <row r="69" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="25"/>
-      <c r="B69"/>
+      <c r="B69" s="90"/>
       <c r="C69" s="25"/>
-      <c r="D69" s="189"/>
-      <c r="E69" s="189"/>
+      <c r="D69" s="166"/>
+      <c r="E69" s="166"/>
       <c r="F69" s="63"/>
       <c r="G69" s="1"/>
       <c r="H69" s="46"/>
       <c r="I69" s="50"/>
       <c r="J69"/>
       <c r="L69"/>
-      <c r="M69" s="56"/>
-      <c r="N69" s="83"/>
-      <c r="O69" s="83"/>
-      <c r="P69" s="57"/>
-      <c r="Q69" s="58"/>
-      <c r="R69" s="58"/>
-      <c r="S69" s="58"/>
-      <c r="T69" s="56"/>
-      <c r="U69" s="56"/>
-    </row>
-    <row r="70" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M69" s="171" t="s">
+        <v>35</v>
+      </c>
+      <c r="N69" s="179"/>
+      <c r="O69" s="179"/>
+      <c r="P69" s="179"/>
+      <c r="Q69" s="179"/>
+      <c r="R69" s="179"/>
+      <c r="S69" s="179"/>
+      <c r="T69" s="179"/>
+      <c r="U69" s="180"/>
+      <c r="V69" s="51"/>
+    </row>
+    <row r="70" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="25"/>
-      <c r="B70" s="90"/>
+      <c r="B70" s="20"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="189"/>
-      <c r="E70" s="189"/>
+      <c r="D70" s="166"/>
+      <c r="E70" s="166"/>
       <c r="F70" s="63"/>
       <c r="G70" s="1"/>
       <c r="H70" s="46"/>
       <c r="I70" s="50"/>
       <c r="J70"/>
-      <c r="L70"/>
-      <c r="M70" s="159" t="s">
-        <v>35</v>
-      </c>
-      <c r="N70" s="160"/>
-      <c r="O70" s="160"/>
-      <c r="P70" s="160"/>
-      <c r="Q70" s="160"/>
-      <c r="R70" s="160"/>
-      <c r="S70" s="160"/>
-      <c r="T70" s="160"/>
-      <c r="U70" s="203"/>
-      <c r="V70" s="51"/>
-    </row>
-    <row r="71" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L70" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="M70" s="130" t="s">
+        <v>55</v>
+      </c>
+      <c r="N70" s="131"/>
+      <c r="O70" s="131"/>
+      <c r="P70" s="131" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q70" s="131"/>
+      <c r="R70" s="131"/>
+      <c r="S70" s="131"/>
+      <c r="T70" s="131" t="s">
+        <v>57</v>
+      </c>
+      <c r="U70" s="132" t="s">
+        <v>60</v>
+      </c>
+      <c r="V70" s="144" t="s">
+        <v>58</v>
+      </c>
+      <c r="W70" s="144" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="25"/>
-      <c r="B71" s="20"/>
+      <c r="B71" s="115"/>
       <c r="C71" s="25"/>
-      <c r="D71" s="189"/>
-      <c r="E71" s="189"/>
+      <c r="D71" s="166"/>
+      <c r="E71" s="166"/>
       <c r="F71" s="63"/>
       <c r="G71" s="1"/>
       <c r="H71" s="46"/>
       <c r="I71" s="50"/>
-      <c r="J71"/>
-      <c r="L71" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="M71" s="130" t="s">
-        <v>55</v>
-      </c>
-      <c r="N71" s="131"/>
-      <c r="O71" s="131"/>
-      <c r="P71" s="131" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q71" s="131"/>
-      <c r="R71" s="131"/>
-      <c r="S71" s="131"/>
-      <c r="T71" s="131" t="s">
-        <v>57</v>
-      </c>
-      <c r="U71" s="132" t="s">
-        <v>60</v>
-      </c>
-      <c r="V71" s="144" t="s">
-        <v>58</v>
-      </c>
-      <c r="W71" s="144" t="s">
-        <v>50</v>
-      </c>
+      <c r="J71" s="23"/>
+      <c r="L71" s="0"/>
+      <c r="M71" s="59"/>
+      <c r="N71" s="60"/>
+      <c r="O71" s="143" t="s">
+        <v>43</v>
+      </c>
+      <c r="P71" s="62"/>
+      <c r="Q71" s="61"/>
+      <c r="R71" s="177" t="s">
+        <v>6</v>
+      </c>
+      <c r="S71" s="177"/>
+      <c r="T71" s="133"/>
+      <c r="U71" s="134"/>
+      <c r="V71" s="51"/>
     </row>
     <row r="72" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="25"/>
-      <c r="B72" s="115"/>
-      <c r="C72" s="25"/>
-      <c r="D72" s="189"/>
-      <c r="E72" s="189"/>
+      <c r="B72" s="51"/>
+      <c r="C72" s="89"/>
+      <c r="D72" s="166"/>
+      <c r="E72" s="166"/>
       <c r="F72" s="63"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="46"/>
-      <c r="I72" s="50"/>
-      <c r="J72" s="23"/>
-      <c r="L72" s="0"/>
-      <c r="M72" s="59"/>
-      <c r="N72" s="60"/>
-      <c r="O72" s="143" t="s">
-        <v>43</v>
-      </c>
-      <c r="P72" s="62"/>
-      <c r="Q72" s="61"/>
-      <c r="R72" s="201" t="s">
-        <v>6</v>
-      </c>
-      <c r="S72" s="201"/>
-      <c r="T72" s="133"/>
-      <c r="U72" s="134"/>
+      <c r="I72" s="115"/>
+      <c r="L72"/>
+      <c r="M72" s="85"/>
+      <c r="N72" s="86"/>
+      <c r="O72" s="18"/>
+      <c r="P72" s="87"/>
+      <c r="Q72" s="56"/>
+      <c r="R72" s="175"/>
+      <c r="S72" s="175"/>
+      <c r="T72" s="65"/>
+      <c r="U72" s="95"/>
       <c r="V72" s="51"/>
     </row>
     <row r="73" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="51"/>
+      <c r="A73" s="49"/>
+      <c r="B73" s="89"/>
       <c r="C73" s="89"/>
-      <c r="D73" s="189"/>
-      <c r="E73" s="189"/>
+      <c r="D73" s="23"/>
+      <c r="E73" s="25"/>
       <c r="F73" s="63"/>
       <c r="I73" s="115"/>
-      <c r="L73"/>
+      <c r="L73" s="45"/>
       <c r="M73" s="85"/>
       <c r="N73" s="86"/>
-      <c r="O73" s="18"/>
+      <c r="O73" s="18" t="s">
+        <v>43</v>
+      </c>
       <c r="P73" s="87"/>
       <c r="Q73" s="56"/>
-      <c r="R73" s="199"/>
-      <c r="S73" s="199"/>
+      <c r="R73" s="175" t="s">
+        <v>10</v>
+      </c>
+      <c r="S73" s="175"/>
       <c r="T73" s="65"/>
       <c r="U73" s="95"/>
       <c r="V73" s="51"/>
     </row>
     <row r="74" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A74" s="49"/>
-      <c r="B74" s="89"/>
-      <c r="C74" s="89"/>
-      <c r="D74" s="23"/>
-      <c r="E74" s="25"/>
-      <c r="F74" s="63"/>
-      <c r="I74" s="115"/>
-      <c r="L74" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12345</t>
-        </is>
-      </c>
-      <c r="M74" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLIENTE UNO</t>
-        </is>
-      </c>
+      <c r="L74" s="45"/>
+      <c r="M74" s="85"/>
       <c r="N74" s="86"/>
-      <c r="O74" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="P74" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F001</t>
-        </is>
-      </c>
+      <c r="O74" s="123"/>
+      <c r="P74" s="87"/>
       <c r="Q74" s="56"/>
-      <c r="R74" s="199" t="s">
-        <v>10</v>
-      </c>
-      <c r="S74" s="199"/>
-      <c r="T74" s="65">
-        <v>150000</v>
-      </c>
-      <c r="U74" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Banco Santander</t>
-        </is>
-      </c>
+      <c r="R74" s="175"/>
+      <c r="S74" s="175"/>
+      <c r="T74" s="65"/>
+      <c r="U74" s="95"/>
       <c r="V74" s="51"/>
     </row>
     <row r="75" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="L75" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">67890</t>
-        </is>
-      </c>
-      <c r="M75" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLIENTE UNO</t>
-        </is>
-      </c>
-      <c r="N75" s="86"/>
-      <c r="O75" s="123"/>
-      <c r="P75" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F001</t>
-        </is>
-      </c>
-      <c r="Q75" s="56"/>
-      <c r="R75" s="199"/>
-      <c r="S75" s="199"/>
-      <c r="T75" s="65">
-        <v>150000</v>
-      </c>
-      <c r="U75" s="95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Banco Santander</t>
-        </is>
-      </c>
+      <c r="L75" s="45"/>
+      <c r="M75" s="137" t="s">
+        <v>61</v>
+      </c>
+      <c r="N75" s="138"/>
+      <c r="O75" s="139"/>
+      <c r="P75" s="140"/>
+      <c r="Q75" s="141"/>
+      <c r="R75" s="176"/>
+      <c r="S75" s="176"/>
+      <c r="T75" s="173"/>
+      <c r="U75" s="174"/>
       <c r="V75" s="51"/>
     </row>
     <row r="76" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
       <c r="L76" s="45"/>
       <c r="M76" s="137" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N76" s="138"/>
       <c r="O76" s="139"/>
       <c r="P76" s="140"/>
       <c r="Q76" s="141"/>
-      <c r="R76" s="200"/>
-      <c r="S76" s="200"/>
-      <c r="T76" s="197"/>
-      <c r="U76" s="198"/>
+      <c r="R76" s="142"/>
+      <c r="S76" s="142"/>
+      <c r="T76" s="173"/>
+      <c r="U76" s="174"/>
       <c r="V76" s="51"/>
     </row>
-    <row r="77" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L77" s="45"/>
-      <c r="M77" s="137" t="s">
-        <v>62</v>
-      </c>
-      <c r="N77" s="138"/>
-      <c r="O77" s="139"/>
-      <c r="P77" s="140"/>
-      <c r="Q77" s="141"/>
-      <c r="R77" s="142"/>
-      <c r="S77" s="142"/>
-      <c r="T77" s="197"/>
-      <c r="U77" s="198"/>
+      <c r="M77" s="94"/>
+      <c r="N77" s="64"/>
+      <c r="O77" s="123"/>
+      <c r="P77" s="87"/>
+      <c r="Q77" s="56"/>
+      <c r="R77" s="56"/>
+      <c r="S77" s="56"/>
+      <c r="T77" s="65"/>
+      <c r="U77" s="95"/>
       <c r="V77" s="51"/>
     </row>
     <row r="78" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="L78" s="45"/>
-      <c r="M78" s="94"/>
-      <c r="N78" s="64"/>
-      <c r="O78" s="123"/>
-      <c r="P78" s="87"/>
-      <c r="Q78" s="56"/>
-      <c r="R78" s="56"/>
-      <c r="S78" s="56"/>
-      <c r="T78" s="65"/>
-      <c r="U78" s="95"/>
+      <c r="M78" s="101" t="s">
+        <v>11</v>
+      </c>
+      <c r="N78" s="102">
+        <f>SUM(N76:N77)</f>
+        <v>0</v>
+      </c>
+      <c r="O78" s="96"/>
+      <c r="P78" s="98"/>
+      <c r="Q78" s="97"/>
+      <c r="R78" s="97"/>
+      <c r="S78" s="97"/>
+      <c r="T78" s="99"/>
+      <c r="U78" s="100"/>
       <c r="V78" s="51"/>
     </row>
-    <row r="79" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="L79" s="45"/>
-      <c r="M79" s="101" t="s">
-        <v>11</v>
-      </c>
-      <c r="N79" s="102">
-        <f>SUM(N77:N78)</f>
-        <v>0</v>
-      </c>
-      <c r="O79" s="96"/>
-      <c r="P79" s="98"/>
-      <c r="Q79" s="97"/>
-      <c r="R79" s="97"/>
-      <c r="S79" s="97"/>
-      <c r="T79" s="99"/>
-      <c r="U79" s="100"/>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M79"/>
+      <c r="O79" s="5"/>
+      <c r="Q79"/>
+      <c r="S79"/>
+      <c r="T79" s="6"/>
       <c r="V79" s="51"/>
     </row>
     <row r="80" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="M80"/>
-      <c r="O80" s="5"/>
-      <c r="Q80"/>
-      <c r="S80"/>
-      <c r="T80" s="6"/>
+      <c r="O80"/>
       <c r="V80" s="51"/>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="O81"/>
+    <row r="81" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="M81" s="23"/>
+      <c r="N81" s="23"/>
+      <c r="O81" s="23"/>
+      <c r="P81" s="23"/>
+      <c r="Q81" s="23"/>
       <c r="V81" s="51"/>
     </row>
     <row r="82" spans="13:22" x14ac:dyDescent="0.3">
-      <c r="M82" s="23"/>
-      <c r="N82" s="23"/>
-      <c r="O82" s="23"/>
-      <c r="P82" s="23"/>
-      <c r="Q82" s="23"/>
       <c r="V82" s="51"/>
     </row>
     <row r="83" spans="13:22" x14ac:dyDescent="0.3">
@@ -4293,7 +4130,7 @@
     <row r="96" spans="13:22" x14ac:dyDescent="0.3">
       <c r="V96" s="51"/>
     </row>
-    <row r="97" spans="13:22" x14ac:dyDescent="0.3">
+    <row r="97" spans="22:22" x14ac:dyDescent="0.3">
       <c r="V97" s="51"/>
     </row>
     <row r="98" spans="22:22" x14ac:dyDescent="0.3">
@@ -4341,53 +4178,19 @@
     <row r="112" spans="22:22" x14ac:dyDescent="0.3">
       <c r="V112" s="51"/>
     </row>
-    <row r="113" spans="22:22" x14ac:dyDescent="0.3">
-      <c r="V113" s="51"/>
-    </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="M68:O68"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="M66:N66"/>
-    <mergeCell ref="T77:U77"/>
-    <mergeCell ref="R75:S75"/>
-    <mergeCell ref="R76:S76"/>
-    <mergeCell ref="R72:S72"/>
-    <mergeCell ref="R74:S74"/>
-    <mergeCell ref="R73:S73"/>
-    <mergeCell ref="T76:U76"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="M70:U70"/>
-    <mergeCell ref="R68:S68"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="P68:Q68"/>
-    <mergeCell ref="T68:U68"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:S33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:S34"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="O32:P32"/>
     <mergeCell ref="M22:U22"/>
     <mergeCell ref="Q26:S26"/>
     <mergeCell ref="O29:P29"/>
@@ -4404,18 +4207,49 @@
     <mergeCell ref="N23:S23"/>
     <mergeCell ref="N24:S24"/>
     <mergeCell ref="T25:U25"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="Q32:S32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="M69:U69"/>
+    <mergeCell ref="R67:S67"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="P67:Q67"/>
+    <mergeCell ref="T67:U67"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="R74:S74"/>
+    <mergeCell ref="R75:S75"/>
+    <mergeCell ref="R71:S71"/>
+    <mergeCell ref="R73:S73"/>
+    <mergeCell ref="R72:S72"/>
+    <mergeCell ref="T75:U75"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="M67:O67"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D51:E51"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>